<commit_message>
Atualiza planilha Display Aramado G
</commit_message>
<xml_diff>
--- a/planilhas/LISTA DE PROCESSO DISPLAY ARAMADO G.xlsx
+++ b/planilhas/LISTA DE PROCESSO DISPLAY ARAMADO G.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\PROJETOS EM ANDAMENTO\PAINEL DE CONTROLE MTECH\PROGRAMAS\PROJETOS  - PAINEL PRODUÇÃO\planilhas\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\PROJETOS EM ANDAMENTO\PAINEL DE CONTROLE MTECH\PROGRAMAS\PROJETOS---BACKEND-IA\planilhas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E19B96C2-72D5-4222-B092-90A4055B0C63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A71647D-6251-41BD-8B70-ACB9398669D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="65">
   <si>
     <t>CLIENTE</t>
   </si>
@@ -162,9 +162,6 @@
   </si>
   <si>
     <t>0,75 Nest 17</t>
-  </si>
-  <si>
-    <t>0,75 Nest 18</t>
   </si>
   <si>
     <t>2,65mm Nest 1</t>
@@ -241,7 +238,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="169" formatCode="0.000000"/>
+    <numFmt numFmtId="164" formatCode="0.000000"/>
   </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
@@ -274,7 +271,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -555,7 +552,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F54"/>
+  <dimension ref="A1:F53"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24.85546875" bestFit="1" customWidth="1"/>
@@ -621,7 +618,7 @@
         <v>22</v>
       </c>
       <c r="E3" s="1">
-        <f t="shared" ref="E3:E29" si="0">F3/1198</f>
+        <f t="shared" ref="E3:E28" si="0">F3/1198</f>
         <v>0.4991652754590985</v>
       </c>
       <c r="F3">
@@ -769,10 +766,10 @@
       </c>
       <c r="E10" s="1">
         <f t="shared" si="0"/>
-        <v>6.3439065108514187E-2</v>
+        <v>6.0934891485809682E-2</v>
       </c>
       <c r="F10">
-        <v>76</v>
+        <v>73</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
@@ -790,10 +787,10 @@
       </c>
       <c r="E11" s="1">
         <f t="shared" si="0"/>
-        <v>9.098497495826377E-2</v>
+        <v>4.1736227045075125E-2</v>
       </c>
       <c r="F11">
-        <v>109</v>
+        <v>50</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
@@ -811,10 +808,10 @@
       </c>
       <c r="E12" s="1">
         <f t="shared" si="0"/>
-        <v>6.7612687813021696E-2</v>
+        <v>9.9332220367278803E-2</v>
       </c>
       <c r="F12">
-        <v>81</v>
+        <v>119</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
@@ -832,10 +829,10 @@
       </c>
       <c r="E13" s="1">
         <f t="shared" si="0"/>
-        <v>3.4223706176961605E-2</v>
+        <v>8.3472454090150253E-4</v>
       </c>
       <c r="F13">
-        <v>41</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
@@ -853,10 +850,10 @@
       </c>
       <c r="E14" s="1">
         <f t="shared" si="0"/>
-        <v>8.3472454090150253E-4</v>
+        <v>9.2654424040066782E-2</v>
       </c>
       <c r="F14">
-        <v>1</v>
+        <v>111</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
@@ -874,10 +871,10 @@
       </c>
       <c r="E15" s="1">
         <f t="shared" si="0"/>
-        <v>8.3472454090150253E-4</v>
+        <v>2.5041736227045075E-3</v>
       </c>
       <c r="F15">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
@@ -895,10 +892,10 @@
       </c>
       <c r="E16" s="1">
         <f t="shared" si="0"/>
-        <v>8.3472454090150253E-4</v>
+        <v>6.6777963272120202E-3</v>
       </c>
       <c r="F16">
-        <v>1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
@@ -916,10 +913,10 @@
       </c>
       <c r="E17" s="1">
         <f t="shared" si="0"/>
-        <v>4.006677796327212E-2</v>
+        <v>3.6727879799666109E-2</v>
       </c>
       <c r="F17">
-        <v>48</v>
+        <v>44</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
@@ -937,10 +934,10 @@
       </c>
       <c r="E18" s="1">
         <f t="shared" si="0"/>
-        <v>2.4207011686143573E-2</v>
+        <v>1.4190317195325543E-2</v>
       </c>
       <c r="F18">
-        <v>29</v>
+        <v>17</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
@@ -958,10 +955,10 @@
       </c>
       <c r="E19" s="1">
         <f t="shared" si="0"/>
-        <v>4.757929883138564E-2</v>
+        <v>0.1310517529215359</v>
       </c>
       <c r="F19">
-        <v>57</v>
+        <v>157</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
@@ -979,10 +976,10 @@
       </c>
       <c r="E20" s="1">
         <f t="shared" si="0"/>
-        <v>2.0868113522537562E-2</v>
+        <v>8.3472454090150253E-4</v>
       </c>
       <c r="F20">
-        <v>25</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
@@ -1000,10 +997,10 @@
       </c>
       <c r="E21" s="1">
         <f t="shared" si="0"/>
-        <v>1.0851419031719533E-2</v>
+        <v>8.3472454090150253E-4</v>
       </c>
       <c r="F21">
-        <v>13</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
@@ -1021,10 +1018,10 @@
       </c>
       <c r="E22" s="1">
         <f t="shared" si="0"/>
-        <v>2.337228714524207E-2</v>
+        <v>2.5041736227045075E-3</v>
       </c>
       <c r="F22">
-        <v>28</v>
+        <v>3</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
@@ -1042,10 +1039,10 @@
       </c>
       <c r="E23" s="1">
         <f t="shared" si="0"/>
-        <v>2.0868113522537562E-2</v>
+        <v>8.3472454090150253E-4</v>
       </c>
       <c r="F23">
-        <v>25</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
@@ -1063,10 +1060,10 @@
       </c>
       <c r="E24" s="1">
         <f t="shared" si="0"/>
-        <v>4.340567612687813E-2</v>
+        <v>8.3472454090150246E-3</v>
       </c>
       <c r="F24">
-        <v>52</v>
+        <v>10</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
@@ -1084,10 +1081,10 @@
       </c>
       <c r="E25" s="1">
         <f t="shared" si="0"/>
-        <v>8.3472454090150253E-4</v>
+        <v>1.4190317195325543E-2</v>
       </c>
       <c r="F25">
-        <v>1</v>
+        <v>17</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
@@ -1105,10 +1102,10 @@
       </c>
       <c r="E26" s="1">
         <f t="shared" si="0"/>
-        <v>2.4207011686143573E-2</v>
+        <v>8.3472454090150253E-4</v>
       </c>
       <c r="F26">
-        <v>29</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
@@ -1126,10 +1123,10 @@
       </c>
       <c r="E27" s="1">
         <f t="shared" si="0"/>
-        <v>8.3472454090150253E-4</v>
+        <v>5.008347245409015E-3</v>
       </c>
       <c r="F27">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
@@ -1147,10 +1144,10 @@
       </c>
       <c r="E28" s="1">
         <f t="shared" si="0"/>
-        <v>5.008347245409015E-3</v>
+        <v>8.3472454090150253E-4</v>
       </c>
       <c r="F28">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
@@ -1161,17 +1158,16 @@
         <v>20</v>
       </c>
       <c r="C29" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D29" t="s">
         <v>44</v>
       </c>
-      <c r="E29" s="1">
-        <f t="shared" si="0"/>
-        <v>8.3472454090150253E-4</v>
+      <c r="E29">
+        <v>2</v>
       </c>
       <c r="F29">
-        <v>1</v>
+        <v>2396</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
@@ -1202,16 +1198,16 @@
         <v>20</v>
       </c>
       <c r="C31" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D31" t="s">
         <v>46</v>
       </c>
       <c r="E31">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F31">
-        <v>2396</v>
+        <v>1198</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
@@ -1228,10 +1224,10 @@
         <v>47</v>
       </c>
       <c r="E32">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F32">
-        <v>1198</v>
+        <v>2396</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
@@ -1242,16 +1238,16 @@
         <v>20</v>
       </c>
       <c r="C33" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D33" t="s">
         <v>48</v>
       </c>
       <c r="E33">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="F33">
-        <v>2396</v>
+        <v>9584</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
@@ -1262,16 +1258,16 @@
         <v>20</v>
       </c>
       <c r="C34" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D34" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="E34">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="F34">
-        <v>9584</v>
+        <v>1198</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
@@ -1282,16 +1278,16 @@
         <v>20</v>
       </c>
       <c r="C35" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D35" t="s">
-        <v>47</v>
+        <v>18</v>
       </c>
       <c r="E35">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F35">
-        <v>1198</v>
+        <v>4792</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
@@ -1305,7 +1301,7 @@
         <v>11</v>
       </c>
       <c r="D36" t="s">
-        <v>18</v>
+        <v>49</v>
       </c>
       <c r="E36">
         <v>4</v>
@@ -1348,10 +1344,10 @@
         <v>51</v>
       </c>
       <c r="E38">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F38">
-        <v>4792</v>
+        <v>2396</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
@@ -1368,10 +1364,10 @@
         <v>52</v>
       </c>
       <c r="E39">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F39">
-        <v>2396</v>
+        <v>1198</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
@@ -1388,10 +1384,10 @@
         <v>53</v>
       </c>
       <c r="E40">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F40">
-        <v>1198</v>
+        <v>2396</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
@@ -1442,16 +1438,16 @@
         <v>20</v>
       </c>
       <c r="C43" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D43" t="s">
         <v>56</v>
       </c>
       <c r="E43">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F43">
-        <v>2396</v>
+        <v>1198</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
@@ -1525,13 +1521,13 @@
         <v>12</v>
       </c>
       <c r="D47" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="E47">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F47">
-        <v>1198</v>
+        <v>4792</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
@@ -1545,13 +1541,13 @@
         <v>12</v>
       </c>
       <c r="D48" t="s">
-        <v>49</v>
+        <v>60</v>
       </c>
       <c r="E48">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F48">
-        <v>4792</v>
+        <v>1198</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
@@ -1585,7 +1581,7 @@
         <v>12</v>
       </c>
       <c r="D50" t="s">
-        <v>62</v>
+        <v>46</v>
       </c>
       <c r="E50">
         <v>1</v>
@@ -1605,7 +1601,7 @@
         <v>12</v>
       </c>
       <c r="D51" t="s">
-        <v>47</v>
+        <v>62</v>
       </c>
       <c r="E51">
         <v>1</v>
@@ -1651,26 +1647,6 @@
         <v>1</v>
       </c>
       <c r="F53">
-        <v>1198</v>
-      </c>
-    </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A54" t="s">
-        <v>19</v>
-      </c>
-      <c r="B54" t="s">
-        <v>20</v>
-      </c>
-      <c r="C54" t="s">
-        <v>12</v>
-      </c>
-      <c r="D54" t="s">
-        <v>65</v>
-      </c>
-      <c r="E54">
-        <v>1</v>
-      </c>
-      <c r="F54">
         <v>1198</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Adiciona lancamentos de pintura
</commit_message>
<xml_diff>
--- a/planilhas/LISTA DE PROCESSO DISPLAY ARAMADO G.xlsx
+++ b/planilhas/LISTA DE PROCESSO DISPLAY ARAMADO G.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\PROJETOS EM ANDAMENTO\PAINEL DE CONTROLE MTECH\PROGRAMAS\PROJETOS---BACKEND-IA\planilhas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A71647D-6251-41BD-8B70-ACB9398669D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A5EC2A2-AFFC-4FD1-9CD0-FAD22FBBF52E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="278" uniqueCount="81">
   <si>
     <t>CLIENTE</t>
   </si>
@@ -231,6 +231,54 @@
   </si>
   <si>
     <t>Apoio Rodizio</t>
+  </si>
+  <si>
+    <t>0,75 Nest 1 AJUSTADA</t>
+  </si>
+  <si>
+    <t>0,75 Nest 2 AJUSTADA</t>
+  </si>
+  <si>
+    <t>0,75 Nest 3 AJUSTADA</t>
+  </si>
+  <si>
+    <t>0,75 Nest 4 AJUSTADA</t>
+  </si>
+  <si>
+    <t>0,75 Nest 5 AJUSTADA</t>
+  </si>
+  <si>
+    <t>0,75 Nest 6 AJUSTADA</t>
+  </si>
+  <si>
+    <t>0,75 Nest 7 AJUSTADA</t>
+  </si>
+  <si>
+    <t>0,75 Nest 8 AJUSTADA</t>
+  </si>
+  <si>
+    <t>0,75 Nest 9 AJUSTADA</t>
+  </si>
+  <si>
+    <t>0,75 Nest 10 AJUSTADA</t>
+  </si>
+  <si>
+    <t>0,75 Nest 11 AJUSTADA</t>
+  </si>
+  <si>
+    <t>0,75 Nest 12 AJUSTADA</t>
+  </si>
+  <si>
+    <t>0,75 Nest 13 AJUSTADA</t>
+  </si>
+  <si>
+    <t>0,75 Nest 14 AJUSTADA</t>
+  </si>
+  <si>
+    <t>0,75 Nest 15 AJUSTADA</t>
+  </si>
+  <si>
+    <t>0,75 Nest 16 AJUSTADA</t>
   </si>
 </sst>
 </file>
@@ -552,7 +600,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F53"/>
+  <dimension ref="A1:F69"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24.85546875" bestFit="1" customWidth="1"/>
@@ -1650,6 +1698,342 @@
         <v>1198</v>
       </c>
     </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>19</v>
+      </c>
+      <c r="B54" t="s">
+        <v>20</v>
+      </c>
+      <c r="C54" t="s">
+        <v>13</v>
+      </c>
+      <c r="D54" t="s">
+        <v>65</v>
+      </c>
+      <c r="E54">
+        <f>F54/1198</f>
+        <v>3.6727879799666109E-2</v>
+      </c>
+      <c r="F54">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>19</v>
+      </c>
+      <c r="B55" t="s">
+        <v>20</v>
+      </c>
+      <c r="C55" t="s">
+        <v>13</v>
+      </c>
+      <c r="D55" t="s">
+        <v>66</v>
+      </c>
+      <c r="E55">
+        <f t="shared" ref="E55:E69" si="1">F55/1198</f>
+        <v>8.3472454090150253E-4</v>
+      </c>
+      <c r="F55">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>19</v>
+      </c>
+      <c r="B56" t="s">
+        <v>20</v>
+      </c>
+      <c r="C56" t="s">
+        <v>13</v>
+      </c>
+      <c r="D56" t="s">
+        <v>67</v>
+      </c>
+      <c r="E56">
+        <f t="shared" si="1"/>
+        <v>8.4307178631051749E-2</v>
+      </c>
+      <c r="F56">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>19</v>
+      </c>
+      <c r="B57" t="s">
+        <v>20</v>
+      </c>
+      <c r="C57" t="s">
+        <v>13</v>
+      </c>
+      <c r="D57" t="s">
+        <v>68</v>
+      </c>
+      <c r="E57">
+        <f t="shared" si="1"/>
+        <v>2.337228714524207E-2</v>
+      </c>
+      <c r="F57">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>19</v>
+      </c>
+      <c r="B58" t="s">
+        <v>20</v>
+      </c>
+      <c r="C58" t="s">
+        <v>13</v>
+      </c>
+      <c r="D58" t="s">
+        <v>69</v>
+      </c>
+      <c r="E58">
+        <f t="shared" si="1"/>
+        <v>0.10517529215358931</v>
+      </c>
+      <c r="F58">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>19</v>
+      </c>
+      <c r="B59" t="s">
+        <v>20</v>
+      </c>
+      <c r="C59" t="s">
+        <v>13</v>
+      </c>
+      <c r="D59" t="s">
+        <v>70</v>
+      </c>
+      <c r="E59">
+        <f t="shared" si="1"/>
+        <v>1.6694490818030051E-3</v>
+      </c>
+      <c r="F59">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>19</v>
+      </c>
+      <c r="B60" t="s">
+        <v>20</v>
+      </c>
+      <c r="C60" t="s">
+        <v>13</v>
+      </c>
+      <c r="D60" t="s">
+        <v>71</v>
+      </c>
+      <c r="E60">
+        <f t="shared" si="1"/>
+        <v>7.5125208681135229E-3</v>
+      </c>
+      <c r="F60">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>19</v>
+      </c>
+      <c r="B61" t="s">
+        <v>20</v>
+      </c>
+      <c r="C61" t="s">
+        <v>13</v>
+      </c>
+      <c r="D61" t="s">
+        <v>72</v>
+      </c>
+      <c r="E61">
+        <f t="shared" si="1"/>
+        <v>8.3472454090150253E-4</v>
+      </c>
+      <c r="F61">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>19</v>
+      </c>
+      <c r="B62" t="s">
+        <v>20</v>
+      </c>
+      <c r="C62" t="s">
+        <v>13</v>
+      </c>
+      <c r="D62" t="s">
+        <v>73</v>
+      </c>
+      <c r="E62">
+        <f t="shared" si="1"/>
+        <v>8.3472454090150253E-4</v>
+      </c>
+      <c r="F62">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>19</v>
+      </c>
+      <c r="B63" t="s">
+        <v>20</v>
+      </c>
+      <c r="C63" t="s">
+        <v>13</v>
+      </c>
+      <c r="D63" t="s">
+        <v>74</v>
+      </c>
+      <c r="E63">
+        <f t="shared" si="1"/>
+        <v>1.6694490818030051E-3</v>
+      </c>
+      <c r="F63">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>19</v>
+      </c>
+      <c r="B64" t="s">
+        <v>20</v>
+      </c>
+      <c r="C64" t="s">
+        <v>13</v>
+      </c>
+      <c r="D64" t="s">
+        <v>75</v>
+      </c>
+      <c r="E64">
+        <f t="shared" si="1"/>
+        <v>1.001669449081803E-2</v>
+      </c>
+      <c r="F64">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>19</v>
+      </c>
+      <c r="B65" t="s">
+        <v>20</v>
+      </c>
+      <c r="C65" t="s">
+        <v>13</v>
+      </c>
+      <c r="D65" t="s">
+        <v>76</v>
+      </c>
+      <c r="E65">
+        <f t="shared" si="1"/>
+        <v>1.6694490818030051E-3</v>
+      </c>
+      <c r="F65">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>19</v>
+      </c>
+      <c r="B66" t="s">
+        <v>20</v>
+      </c>
+      <c r="C66" t="s">
+        <v>13</v>
+      </c>
+      <c r="D66" t="s">
+        <v>77</v>
+      </c>
+      <c r="E66">
+        <f t="shared" si="1"/>
+        <v>5.008347245409015E-3</v>
+      </c>
+      <c r="F66">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>19</v>
+      </c>
+      <c r="B67" t="s">
+        <v>20</v>
+      </c>
+      <c r="C67" t="s">
+        <v>13</v>
+      </c>
+      <c r="D67" t="s">
+        <v>78</v>
+      </c>
+      <c r="E67">
+        <f t="shared" si="1"/>
+        <v>2.1702838063439065E-2</v>
+      </c>
+      <c r="F67">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>19</v>
+      </c>
+      <c r="B68" t="s">
+        <v>20</v>
+      </c>
+      <c r="C68" t="s">
+        <v>13</v>
+      </c>
+      <c r="D68" t="s">
+        <v>79</v>
+      </c>
+      <c r="E68">
+        <f t="shared" si="1"/>
+        <v>3.0050083472454091E-2</v>
+      </c>
+      <c r="F68">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>19</v>
+      </c>
+      <c r="B69" t="s">
+        <v>20</v>
+      </c>
+      <c r="C69" t="s">
+        <v>13</v>
+      </c>
+      <c r="D69" t="s">
+        <v>80</v>
+      </c>
+      <c r="E69">
+        <f t="shared" si="1"/>
+        <v>8.3472454090150253E-4</v>
+      </c>
+      <c r="F69">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Adiciona IDs e QR Codes para processos de produção
</commit_message>
<xml_diff>
--- a/planilhas/LISTA DE PROCESSO DISPLAY ARAMADO G.xlsx
+++ b/planilhas/LISTA DE PROCESSO DISPLAY ARAMADO G.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\PROJETOS EM ANDAMENTO\PAINEL DE CONTROLE MTECH\PROGRAMAS\PROJETOS---BACKEND-IA\planilhas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A5EC2A2-AFFC-4FD1-9CD0-FAD22FBBF52E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A38E9509-7F92-43E1-9339-95AED4DD60F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,9 +17,6 @@
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
@@ -36,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="278" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="347" uniqueCount="150">
   <si>
     <t>CLIENTE</t>
   </si>
@@ -56,156 +53,156 @@
     <t>QNT TOTAL</t>
   </si>
   <si>
+    <t>JDE COFFEE</t>
+  </si>
+  <si>
+    <t>DISPLAY ARAMADO G</t>
+  </si>
+  <si>
     <t>Laser Tube</t>
   </si>
   <si>
+    <t>20X20 Nest 1</t>
+  </si>
+  <si>
+    <t>20X20 Nest 2</t>
+  </si>
+  <si>
+    <t>20X20 Nest 3</t>
+  </si>
+  <si>
+    <t>20X20 Nest 4</t>
+  </si>
+  <si>
+    <t>20X20 Nest 5</t>
+  </si>
+  <si>
+    <t>20X20 Nest 6</t>
+  </si>
+  <si>
+    <t>20X20 Nest 7</t>
+  </si>
+  <si>
+    <t>20X20 Nest 8</t>
+  </si>
+  <si>
+    <t>Laser Chapa</t>
+  </si>
+  <si>
+    <t>0,75 Nest 1</t>
+  </si>
+  <si>
+    <t>0,75 Nest 2</t>
+  </si>
+  <si>
+    <t>0,75 Nest 3</t>
+  </si>
+  <si>
+    <t>0,75 Nest 4</t>
+  </si>
+  <si>
+    <t>0,75 Nest 5</t>
+  </si>
+  <si>
+    <t>0,75 Nest 6</t>
+  </si>
+  <si>
+    <t>0,75 Nest 7</t>
+  </si>
+  <si>
+    <t>0,75 Nest 8</t>
+  </si>
+  <si>
+    <t>0,75 Nest 9</t>
+  </si>
+  <si>
+    <t>0,75 Nest 10</t>
+  </si>
+  <si>
+    <t>0,75 Nest 11</t>
+  </si>
+  <si>
+    <t>0,75 Nest 12</t>
+  </si>
+  <si>
+    <t>0,75 Nest 13</t>
+  </si>
+  <si>
+    <t>0,75 Nest 14</t>
+  </si>
+  <si>
+    <t>0,75 Nest 15</t>
+  </si>
+  <si>
+    <t>0,75 Nest 16</t>
+  </si>
+  <si>
+    <t>0,75 Nest 17</t>
+  </si>
+  <si>
+    <t>2,65mm Nest 1</t>
+  </si>
+  <si>
+    <t>2,65mm Nest 2</t>
+  </si>
+  <si>
+    <t>Guilhotina</t>
+  </si>
+  <si>
+    <t>CORPO ◄J► 120 mm</t>
+  </si>
+  <si>
+    <t>CORPO ◄J► 210 mm</t>
+  </si>
+  <si>
     <t>Serra</t>
   </si>
   <si>
-    <t>Guilhotina</t>
+    <t>Parachoque</t>
+  </si>
+  <si>
+    <t>Tubo Testeira e Corpo 360mm</t>
   </si>
   <si>
     <t>Dobradeira de Arames</t>
   </si>
   <si>
+    <t>Arame Bdj</t>
+  </si>
+  <si>
     <t>Dobradeira de Tubos</t>
   </si>
   <si>
     <t>Dobradeira de Chapas</t>
   </si>
   <si>
+    <t>Bandeja</t>
+  </si>
+  <si>
+    <t>Bandeja Amassamento</t>
+  </si>
+  <si>
+    <t>J 786mm Lateral</t>
+  </si>
+  <si>
+    <t>J 1200mm Traseira</t>
+  </si>
+  <si>
+    <t>J 400mm Base</t>
+  </si>
+  <si>
+    <t>J 120mm Base</t>
+  </si>
+  <si>
+    <t>J 210mm Base</t>
+  </si>
+  <si>
+    <t>Encaixe Tubo Testeira</t>
+  </si>
+  <si>
     <t>Solda Mig</t>
   </si>
   <si>
-    <t>Laser Chapa</t>
-  </si>
-  <si>
-    <t>0,75 Nest 1</t>
-  </si>
-  <si>
-    <t>0,75 Nest 2</t>
-  </si>
-  <si>
-    <t>0,75 Nest 3</t>
-  </si>
-  <si>
-    <t>0,75 Nest 4</t>
-  </si>
-  <si>
-    <t>Bandeja</t>
-  </si>
-  <si>
-    <t>JDE COFFEE</t>
-  </si>
-  <si>
-    <t>DISPLAY ARAMADO G</t>
-  </si>
-  <si>
-    <t>20X20 Nest 1</t>
-  </si>
-  <si>
-    <t>20X20 Nest 2</t>
-  </si>
-  <si>
-    <t>20X20 Nest 3</t>
-  </si>
-  <si>
-    <t>20X20 Nest 4</t>
-  </si>
-  <si>
-    <t>20X20 Nest 5</t>
-  </si>
-  <si>
-    <t>20X20 Nest 6</t>
-  </si>
-  <si>
-    <t>20X20 Nest 7</t>
-  </si>
-  <si>
-    <t>20X20 Nest 8</t>
-  </si>
-  <si>
-    <t>0,75 Nest 5</t>
-  </si>
-  <si>
-    <t>0,75 Nest 6</t>
-  </si>
-  <si>
-    <t>0,75 Nest 7</t>
-  </si>
-  <si>
-    <t>0,75 Nest 8</t>
-  </si>
-  <si>
-    <t>0,75 Nest 9</t>
-  </si>
-  <si>
-    <t>0,75 Nest 10</t>
-  </si>
-  <si>
-    <t>0,75 Nest 11</t>
-  </si>
-  <si>
-    <t>0,75 Nest 12</t>
-  </si>
-  <si>
-    <t>0,75 Nest 13</t>
-  </si>
-  <si>
-    <t>0,75 Nest 14</t>
-  </si>
-  <si>
-    <t>0,75 Nest 15</t>
-  </si>
-  <si>
-    <t>0,75 Nest 16</t>
-  </si>
-  <si>
-    <t>0,75 Nest 17</t>
-  </si>
-  <si>
-    <t>2,65mm Nest 1</t>
-  </si>
-  <si>
-    <t>2,65mm Nest 2</t>
-  </si>
-  <si>
-    <t>CORPO ◄J► 120 mm</t>
-  </si>
-  <si>
-    <t>CORPO ◄J► 210 mm</t>
-  </si>
-  <si>
-    <t>Parachoque</t>
-  </si>
-  <si>
-    <t>Tubo Testeira e Corpo 360mm</t>
-  </si>
-  <si>
-    <t>Arame Bdj</t>
-  </si>
-  <si>
-    <t>Bandeja Amassamento</t>
-  </si>
-  <si>
-    <t>J 786mm Lateral</t>
-  </si>
-  <si>
-    <t>J 1200mm Traseira</t>
-  </si>
-  <si>
-    <t>J 400mm Base</t>
-  </si>
-  <si>
-    <t>J 120mm Base</t>
-  </si>
-  <si>
-    <t>J 210mm Base</t>
-  </si>
-  <si>
-    <t>Encaixe Tubo Testeira</t>
-  </si>
-  <si>
     <t>Fechamento Base</t>
   </si>
   <si>
@@ -279,6 +276,213 @@
   </si>
   <si>
     <t>0,75 Nest 16 AJUSTADA</t>
+  </si>
+  <si>
+    <t>PROCESSO_ID</t>
+  </si>
+  <si>
+    <t>000030</t>
+  </si>
+  <si>
+    <t>000031</t>
+  </si>
+  <si>
+    <t>000032</t>
+  </si>
+  <si>
+    <t>000033</t>
+  </si>
+  <si>
+    <t>000034</t>
+  </si>
+  <si>
+    <t>000035</t>
+  </si>
+  <si>
+    <t>000036</t>
+  </si>
+  <si>
+    <t>000037</t>
+  </si>
+  <si>
+    <t>000038</t>
+  </si>
+  <si>
+    <t>000039</t>
+  </si>
+  <si>
+    <t>000040</t>
+  </si>
+  <si>
+    <t>000041</t>
+  </si>
+  <si>
+    <t>000042</t>
+  </si>
+  <si>
+    <t>000043</t>
+  </si>
+  <si>
+    <t>000044</t>
+  </si>
+  <si>
+    <t>000045</t>
+  </si>
+  <si>
+    <t>000046</t>
+  </si>
+  <si>
+    <t>000047</t>
+  </si>
+  <si>
+    <t>000048</t>
+  </si>
+  <si>
+    <t>000049</t>
+  </si>
+  <si>
+    <t>000050</t>
+  </si>
+  <si>
+    <t>000051</t>
+  </si>
+  <si>
+    <t>000052</t>
+  </si>
+  <si>
+    <t>000053</t>
+  </si>
+  <si>
+    <t>000054</t>
+  </si>
+  <si>
+    <t>000055</t>
+  </si>
+  <si>
+    <t>000056</t>
+  </si>
+  <si>
+    <t>000057</t>
+  </si>
+  <si>
+    <t>000058</t>
+  </si>
+  <si>
+    <t>000059</t>
+  </si>
+  <si>
+    <t>000060</t>
+  </si>
+  <si>
+    <t>000061</t>
+  </si>
+  <si>
+    <t>000062</t>
+  </si>
+  <si>
+    <t>000063</t>
+  </si>
+  <si>
+    <t>000064</t>
+  </si>
+  <si>
+    <t>000065</t>
+  </si>
+  <si>
+    <t>000066</t>
+  </si>
+  <si>
+    <t>000067</t>
+  </si>
+  <si>
+    <t>000068</t>
+  </si>
+  <si>
+    <t>000069</t>
+  </si>
+  <si>
+    <t>000070</t>
+  </si>
+  <si>
+    <t>000071</t>
+  </si>
+  <si>
+    <t>000072</t>
+  </si>
+  <si>
+    <t>000073</t>
+  </si>
+  <si>
+    <t>000074</t>
+  </si>
+  <si>
+    <t>000075</t>
+  </si>
+  <si>
+    <t>000076</t>
+  </si>
+  <si>
+    <t>000077</t>
+  </si>
+  <si>
+    <t>000078</t>
+  </si>
+  <si>
+    <t>000079</t>
+  </si>
+  <si>
+    <t>000080</t>
+  </si>
+  <si>
+    <t>000081</t>
+  </si>
+  <si>
+    <t>000082</t>
+  </si>
+  <si>
+    <t>000083</t>
+  </si>
+  <si>
+    <t>000084</t>
+  </si>
+  <si>
+    <t>000085</t>
+  </si>
+  <si>
+    <t>000086</t>
+  </si>
+  <si>
+    <t>000087</t>
+  </si>
+  <si>
+    <t>000088</t>
+  </si>
+  <si>
+    <t>000089</t>
+  </si>
+  <si>
+    <t>000090</t>
+  </si>
+  <si>
+    <t>000091</t>
+  </si>
+  <si>
+    <t>000092</t>
+  </si>
+  <si>
+    <t>000093</t>
+  </si>
+  <si>
+    <t>000094</t>
+  </si>
+  <si>
+    <t>000095</t>
+  </si>
+  <si>
+    <t>000096</t>
+  </si>
+  <si>
+    <t>000097</t>
   </si>
 </sst>
 </file>
@@ -293,8 +497,6 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -317,9 +519,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -380,74 +585,14 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="Yu Gothic Light"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线 Light"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:latin typeface="Calibri Light"/>
+        <a:ea typeface="Calibri Light"/>
+        <a:cs typeface="Calibri Light"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="Yu Gothic"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface="Calibri"/>
+        <a:cs typeface="Calibri"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -459,23 +604,23 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
+                <a:tint val="67000"/>
                 <a:lumMod val="110000"/>
                 <a:satMod val="105000"/>
-                <a:tint val="67000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="50000">
               <a:schemeClr val="phClr">
+                <a:tint val="73000"/>
                 <a:lumMod val="105000"/>
                 <a:satMod val="103000"/>
-                <a:tint val="73000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
+                <a:tint val="81000"/>
                 <a:lumMod val="105000"/>
                 <a:satMod val="109000"/>
-                <a:tint val="81000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -485,23 +630,23 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
+                <a:tint val="94000"/>
+                <a:lumMod val="102000"/>
                 <a:satMod val="103000"/>
-                <a:lumMod val="102000"/>
-                <a:tint val="94000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="50000">
               <a:schemeClr val="phClr">
+                <a:shade val="100000"/>
+                <a:lumMod val="100000"/>
                 <a:satMod val="110000"/>
-                <a:lumMod val="100000"/>
-                <a:shade val="100000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
+                <a:shade val="78000"/>
                 <a:lumMod val="99000"/>
                 <a:satMod val="120000"/>
-                <a:shade val="78000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -509,26 +654,23 @@
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="6350">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="12700">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
-        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="19050">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
@@ -563,17 +705,17 @@
             <a:gs pos="0">
               <a:schemeClr val="phClr">
                 <a:tint val="93000"/>
-                <a:satMod val="150000"/>
                 <a:shade val="98000"/>
                 <a:lumMod val="102000"/>
+                <a:satMod val="150000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="50000">
               <a:schemeClr val="phClr">
                 <a:tint val="98000"/>
-                <a:satMod val="130000"/>
                 <a:shade val="90000"/>
                 <a:lumMod val="103000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
@@ -590,28 +732,24 @@
   </a:themeElements>
   <a:objectDefaults/>
   <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
-    </a:ext>
-  </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F69"/>
+  <dimension ref="A1:G69"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="24.85546875" customWidth="1"/>
     <col min="2" max="2" width="32.7109375" customWidth="1"/>
     <col min="3" max="3" width="27.85546875" customWidth="1"/>
     <col min="4" max="4" width="38.85546875" customWidth="1"/>
-    <col min="5" max="5" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.5703125" customWidth="1"/>
     <col min="6" max="6" width="12.28515625" customWidth="1"/>
+    <col min="7" max="7" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -630,19 +768,22 @@
       <c r="F1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G1" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="B2" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D2" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="E2" s="1">
         <f>F2/1198</f>
@@ -651,19 +792,22 @@
       <c r="F2">
         <v>399</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G2" s="2" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="B3" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C3" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D3" t="s">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="E3" s="1">
         <f t="shared" ref="E3:E28" si="0">F3/1198</f>
@@ -672,19 +816,22 @@
       <c r="F3">
         <v>598</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G3" s="2" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="B4" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C4" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D4" t="s">
-        <v>23</v>
+        <v>11</v>
       </c>
       <c r="E4" s="1">
         <f t="shared" si="0"/>
@@ -693,19 +840,22 @@
       <c r="F4">
         <v>97</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G4" s="2" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="B5" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C5" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D5" t="s">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="E5" s="1">
         <f t="shared" si="0"/>
@@ -714,19 +864,22 @@
       <c r="F5">
         <v>221</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G5" s="2" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="B6" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C6" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D6" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="E6" s="1">
         <f t="shared" si="0"/>
@@ -735,19 +888,22 @@
       <c r="F6">
         <v>243</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G6" s="2" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C7" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D7" t="s">
-        <v>26</v>
+        <v>14</v>
       </c>
       <c r="E7" s="1">
         <f t="shared" si="0"/>
@@ -756,19 +912,22 @@
       <c r="F7">
         <v>275</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G7" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C8" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D8" t="s">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="E8" s="1">
         <f t="shared" si="0"/>
@@ -777,19 +936,22 @@
       <c r="F8">
         <v>1</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G8" s="2" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="B9" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C9" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D9" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="E9" s="1">
         <f t="shared" si="0"/>
@@ -798,19 +960,22 @@
       <c r="F9">
         <v>1</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G9" s="2" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="B10" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C10" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="D10" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="E10" s="1">
         <f t="shared" si="0"/>
@@ -819,19 +984,22 @@
       <c r="F10">
         <v>73</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G10" s="2" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>6</v>
+      </c>
+      <c r="B11" t="s">
+        <v>7</v>
+      </c>
+      <c r="C11" t="s">
+        <v>17</v>
+      </c>
+      <c r="D11" t="s">
         <v>19</v>
-      </c>
-      <c r="B11" t="s">
-        <v>20</v>
-      </c>
-      <c r="C11" t="s">
-        <v>13</v>
-      </c>
-      <c r="D11" t="s">
-        <v>15</v>
       </c>
       <c r="E11" s="1">
         <f t="shared" si="0"/>
@@ -840,19 +1008,22 @@
       <c r="F11">
         <v>50</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G11" s="2" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="B12" t="s">
+        <v>7</v>
+      </c>
+      <c r="C12" t="s">
+        <v>17</v>
+      </c>
+      <c r="D12" t="s">
         <v>20</v>
-      </c>
-      <c r="C12" t="s">
-        <v>13</v>
-      </c>
-      <c r="D12" t="s">
-        <v>16</v>
       </c>
       <c r="E12" s="1">
         <f t="shared" si="0"/>
@@ -861,19 +1032,22 @@
       <c r="F12">
         <v>119</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G12" s="2" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="B13" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C13" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="D13" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E13" s="1">
         <f t="shared" si="0"/>
@@ -882,19 +1056,22 @@
       <c r="F13">
         <v>1</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G13" s="2" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="B14" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C14" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="D14" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="E14" s="1">
         <f t="shared" si="0"/>
@@ -903,19 +1080,22 @@
       <c r="F14">
         <v>111</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G14" s="2" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="B15" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C15" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="D15" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="E15" s="1">
         <f t="shared" si="0"/>
@@ -924,19 +1104,22 @@
       <c r="F15">
         <v>3</v>
       </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G15" s="2" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="B16" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C16" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="D16" t="s">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="E16" s="1">
         <f t="shared" si="0"/>
@@ -945,19 +1128,22 @@
       <c r="F16">
         <v>8</v>
       </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G16" s="2" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="B17" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C17" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="D17" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="E17" s="1">
         <f t="shared" si="0"/>
@@ -966,19 +1152,22 @@
       <c r="F17">
         <v>44</v>
       </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G17" s="2" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="B18" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C18" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="D18" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="E18" s="1">
         <f t="shared" si="0"/>
@@ -987,19 +1176,22 @@
       <c r="F18">
         <v>17</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G18" s="2" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="B19" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C19" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="D19" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="E19" s="1">
         <f t="shared" si="0"/>
@@ -1008,19 +1200,22 @@
       <c r="F19">
         <v>157</v>
       </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G19" s="2" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="B20" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C20" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="D20" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="E20" s="1">
         <f t="shared" si="0"/>
@@ -1029,19 +1224,22 @@
       <c r="F20">
         <v>1</v>
       </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G20" s="2" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="B21" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C21" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="D21" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="E21" s="1">
         <f t="shared" si="0"/>
@@ -1050,19 +1248,22 @@
       <c r="F21">
         <v>1</v>
       </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G21" s="2" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="B22" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C22" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="D22" t="s">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="E22" s="1">
         <f t="shared" si="0"/>
@@ -1071,19 +1272,22 @@
       <c r="F22">
         <v>3</v>
       </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G22" s="2" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="B23" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C23" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="D23" t="s">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="E23" s="1">
         <f t="shared" si="0"/>
@@ -1092,19 +1296,22 @@
       <c r="F23">
         <v>1</v>
       </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G23" s="2" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="B24" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C24" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="D24" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="E24" s="1">
         <f t="shared" si="0"/>
@@ -1113,19 +1320,22 @@
       <c r="F24">
         <v>10</v>
       </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G24" s="2" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="B25" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C25" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="D25" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="E25" s="1">
         <f t="shared" si="0"/>
@@ -1134,19 +1344,22 @@
       <c r="F25">
         <v>17</v>
       </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G25" s="2" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="B26" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C26" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="D26" t="s">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="E26" s="1">
         <f t="shared" si="0"/>
@@ -1155,19 +1368,22 @@
       <c r="F26">
         <v>1</v>
       </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G26" s="2" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="B27" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C27" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="D27" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="E27" s="1">
         <f t="shared" si="0"/>
@@ -1176,19 +1392,22 @@
       <c r="F27">
         <v>6</v>
       </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G27" s="2" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="B28" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C28" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="D28" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="E28" s="1">
         <f t="shared" si="0"/>
@@ -1197,19 +1416,22 @@
       <c r="F28">
         <v>1</v>
       </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G28" s="2" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="B29" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C29" t="s">
-        <v>8</v>
+        <v>37</v>
       </c>
       <c r="D29" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="E29">
         <v>2</v>
@@ -1217,19 +1439,22 @@
       <c r="F29">
         <v>2396</v>
       </c>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G29" s="2" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="B30" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C30" t="s">
-        <v>8</v>
+        <v>37</v>
       </c>
       <c r="D30" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="E30">
         <v>2</v>
@@ -1237,19 +1462,22 @@
       <c r="F30">
         <v>2396</v>
       </c>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G30" s="2" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="B31" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C31" t="s">
-        <v>7</v>
+        <v>40</v>
       </c>
       <c r="D31" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="E31">
         <v>1</v>
@@ -1257,19 +1485,22 @@
       <c r="F31">
         <v>1198</v>
       </c>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G31" s="2" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="B32" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C32" t="s">
-        <v>7</v>
+        <v>40</v>
       </c>
       <c r="D32" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="E32">
         <v>2</v>
@@ -1277,19 +1508,22 @@
       <c r="F32">
         <v>2396</v>
       </c>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G32" s="2" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="B33" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C33" t="s">
-        <v>9</v>
+        <v>43</v>
       </c>
       <c r="D33" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="E33">
         <v>8</v>
@@ -1297,19 +1531,22 @@
       <c r="F33">
         <v>9584</v>
       </c>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G33" s="2" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="B34" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C34" t="s">
-        <v>10</v>
+        <v>45</v>
       </c>
       <c r="D34" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="E34">
         <v>1</v>
@@ -1317,19 +1554,22 @@
       <c r="F34">
         <v>1198</v>
       </c>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G34" s="2" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="B35" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C35" t="s">
-        <v>11</v>
+        <v>46</v>
       </c>
       <c r="D35" t="s">
-        <v>18</v>
+        <v>47</v>
       </c>
       <c r="E35">
         <v>4</v>
@@ -1337,19 +1577,22 @@
       <c r="F35">
         <v>4792</v>
       </c>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G35" s="2" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="B36" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C36" t="s">
-        <v>11</v>
+        <v>46</v>
       </c>
       <c r="D36" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E36">
         <v>4</v>
@@ -1357,19 +1600,22 @@
       <c r="F36">
         <v>4792</v>
       </c>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G36" s="2" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="B37" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C37" t="s">
-        <v>11</v>
+        <v>46</v>
       </c>
       <c r="D37" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E37">
         <v>4</v>
@@ -1377,19 +1623,22 @@
       <c r="F37">
         <v>4792</v>
       </c>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G37" s="2" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="B38" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C38" t="s">
-        <v>11</v>
+        <v>46</v>
       </c>
       <c r="D38" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E38">
         <v>2</v>
@@ -1397,19 +1646,22 @@
       <c r="F38">
         <v>2396</v>
       </c>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G38" s="2" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="B39" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C39" t="s">
-        <v>11</v>
+        <v>46</v>
       </c>
       <c r="D39" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E39">
         <v>1</v>
@@ -1417,19 +1669,22 @@
       <c r="F39">
         <v>1198</v>
       </c>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G39" s="2" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="B40" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C40" t="s">
-        <v>11</v>
+        <v>46</v>
       </c>
       <c r="D40" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E40">
         <v>2</v>
@@ -1437,19 +1692,22 @@
       <c r="F40">
         <v>2396</v>
       </c>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G40" s="2" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="B41" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C41" t="s">
-        <v>11</v>
+        <v>46</v>
       </c>
       <c r="D41" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E41">
         <v>2</v>
@@ -1457,19 +1715,22 @@
       <c r="F41">
         <v>2396</v>
       </c>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G41" s="2" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="B42" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C42" t="s">
-        <v>11</v>
+        <v>46</v>
       </c>
       <c r="D42" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E42">
         <v>2</v>
@@ -1477,16 +1738,19 @@
       <c r="F42">
         <v>2396</v>
       </c>
-    </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G42" s="2" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="B43" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C43" t="s">
-        <v>12</v>
+        <v>55</v>
       </c>
       <c r="D43" t="s">
         <v>56</v>
@@ -1497,16 +1761,19 @@
       <c r="F43">
         <v>1198</v>
       </c>
-    </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G43" s="2" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="B44" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C44" t="s">
-        <v>12</v>
+        <v>55</v>
       </c>
       <c r="D44" t="s">
         <v>57</v>
@@ -1517,16 +1784,19 @@
       <c r="F44">
         <v>1198</v>
       </c>
-    </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G44" s="2" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="B45" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C45" t="s">
-        <v>12</v>
+        <v>55</v>
       </c>
       <c r="D45" t="s">
         <v>58</v>
@@ -1537,16 +1807,19 @@
       <c r="F45">
         <v>1198</v>
       </c>
-    </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G45" s="2" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="B46" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C46" t="s">
-        <v>12</v>
+        <v>55</v>
       </c>
       <c r="D46" t="s">
         <v>59</v>
@@ -1557,19 +1830,22 @@
       <c r="F46">
         <v>1198</v>
       </c>
-    </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G46" s="2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="B47" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C47" t="s">
-        <v>12</v>
+        <v>55</v>
       </c>
       <c r="D47" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="E47">
         <v>4</v>
@@ -1577,16 +1853,19 @@
       <c r="F47">
         <v>4792</v>
       </c>
-    </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G47" s="2" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="B48" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C48" t="s">
-        <v>12</v>
+        <v>55</v>
       </c>
       <c r="D48" t="s">
         <v>60</v>
@@ -1597,16 +1876,19 @@
       <c r="F48">
         <v>1198</v>
       </c>
-    </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G48" s="2" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="B49" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C49" t="s">
-        <v>12</v>
+        <v>55</v>
       </c>
       <c r="D49" t="s">
         <v>61</v>
@@ -1617,19 +1899,22 @@
       <c r="F49">
         <v>1198</v>
       </c>
-    </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G49" s="2" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="B50" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C50" t="s">
-        <v>12</v>
+        <v>55</v>
       </c>
       <c r="D50" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="E50">
         <v>1</v>
@@ -1637,16 +1922,19 @@
       <c r="F50">
         <v>1198</v>
       </c>
-    </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G50" s="2" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="B51" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C51" t="s">
-        <v>12</v>
+        <v>55</v>
       </c>
       <c r="D51" t="s">
         <v>62</v>
@@ -1657,16 +1945,19 @@
       <c r="F51">
         <v>1198</v>
       </c>
-    </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G51" s="2" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="B52" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C52" t="s">
-        <v>12</v>
+        <v>55</v>
       </c>
       <c r="D52" t="s">
         <v>63</v>
@@ -1677,16 +1968,19 @@
       <c r="F52">
         <v>1198</v>
       </c>
-    </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G52" s="2" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="B53" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C53" t="s">
-        <v>12</v>
+        <v>55</v>
       </c>
       <c r="D53" t="s">
         <v>64</v>
@@ -1697,16 +1991,19 @@
       <c r="F53">
         <v>1198</v>
       </c>
-    </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G53" s="2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="B54" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C54" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="D54" t="s">
         <v>65</v>
@@ -1718,16 +2015,19 @@
       <c r="F54">
         <v>44</v>
       </c>
-    </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G54" s="2" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="B55" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C55" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="D55" t="s">
         <v>66</v>
@@ -1739,16 +2039,19 @@
       <c r="F55">
         <v>1</v>
       </c>
-    </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G55" s="2" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="B56" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C56" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="D56" t="s">
         <v>67</v>
@@ -1760,16 +2063,19 @@
       <c r="F56">
         <v>101</v>
       </c>
-    </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G56" s="2" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="B57" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C57" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="D57" t="s">
         <v>68</v>
@@ -1781,16 +2087,19 @@
       <c r="F57">
         <v>28</v>
       </c>
-    </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G57" s="2" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="B58" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C58" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="D58" t="s">
         <v>69</v>
@@ -1802,16 +2111,19 @@
       <c r="F58">
         <v>126</v>
       </c>
-    </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G58" s="2" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="B59" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C59" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="D59" t="s">
         <v>70</v>
@@ -1823,16 +2135,19 @@
       <c r="F59">
         <v>2</v>
       </c>
-    </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G59" s="2" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="B60" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C60" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="D60" t="s">
         <v>71</v>
@@ -1844,16 +2159,19 @@
       <c r="F60">
         <v>9</v>
       </c>
-    </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G60" s="2" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="B61" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C61" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="D61" t="s">
         <v>72</v>
@@ -1865,16 +2183,19 @@
       <c r="F61">
         <v>1</v>
       </c>
-    </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G61" s="2" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="B62" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C62" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="D62" t="s">
         <v>73</v>
@@ -1886,16 +2207,19 @@
       <c r="F62">
         <v>1</v>
       </c>
-    </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G62" s="2" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="B63" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C63" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="D63" t="s">
         <v>74</v>
@@ -1907,16 +2231,19 @@
       <c r="F63">
         <v>2</v>
       </c>
-    </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G63" s="2" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="B64" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C64" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="D64" t="s">
         <v>75</v>
@@ -1928,16 +2255,19 @@
       <c r="F64">
         <v>12</v>
       </c>
-    </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G64" s="2" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="B65" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C65" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="D65" t="s">
         <v>76</v>
@@ -1949,16 +2279,19 @@
       <c r="F65">
         <v>2</v>
       </c>
-    </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G65" s="2" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="B66" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C66" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="D66" t="s">
         <v>77</v>
@@ -1970,16 +2303,19 @@
       <c r="F66">
         <v>6</v>
       </c>
-    </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G66" s="2" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="B67" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C67" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="D67" t="s">
         <v>78</v>
@@ -1991,16 +2327,19 @@
       <c r="F67">
         <v>26</v>
       </c>
-    </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G67" s="2" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="B68" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C68" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="D68" t="s">
         <v>79</v>
@@ -2012,16 +2351,19 @@
       <c r="F68">
         <v>36</v>
       </c>
-    </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G68" s="2" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="B69" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C69" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="D69" t="s">
         <v>80</v>
@@ -2032,6 +2374,9 @@
       </c>
       <c r="F69">
         <v>1</v>
+      </c>
+      <c r="G69" s="2" t="s">
+        <v>149</v>
       </c>
     </row>
   </sheetData>

</xml_diff>